<commit_message>
Educación temprana (b): narrativa por país (estilo resumen oficial) + enlaces
Para cada país, un párrafo narrativo al estilo del resumen oficial del ILIA (como el de
Trinidad y Tobago): fuentes revisadas, hallazgos de IA/TIC con cita y página, categoría +
puntaje + justificación (por qué no las categorías contiguas), y los enlaces a las fuentes.

- entrega/_narrativas.py: fuente única (párrafos + enlaces por país).
- narrativas_por_pais.md: las 5 narrativas con enlaces.
- INFORME_FINAL_2026-06-06.xlsx: nueva hoja «Narrativa por país» (párrafo + fuentes clicables).
- INFORME_FINAL_2026-06-06.{pdf,docx,html,md} regenerado (18 pp): narrativa integrada tras el
  informe técnico.
- entrega/_build_xlsx.py y _build_pdf.py: enganchan _narrativas.
</commit_message>
<xml_diff>
--- a/data/educacion_temprana/entrega/INFORME_FINAL_2026-06-06.xlsx
+++ b/data/educacion_temprana/entrega/INFORME_FINAL_2026-06-06.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidencia verbatim" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metodología" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Narrativa por país" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$1:$K$1</definedName>
@@ -22,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -52,6 +53,15 @@
       <b val="1"/>
       <color rgb="000B3D6B"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="6">
@@ -108,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -142,6 +152,14 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2858,4 +2876,312 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="118" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Narrativa por país — resumen oficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>España (ES)</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Categoría 5 — 100 puntos</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="170" customHeight="1">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>Análisis</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>Para el subindicador «Educación Temprana en IA» del ILIA 2026 se examinó si la base curricular oficial vigente de España incorpora contenidos de inteligencia artificial o de TIC en la educación secundaria (ESO y Bachillerato). Sobre el marco de la LOMLOE, se revisaron los Reales Decretos de enseñanzas mínimas publicados en el BOE —RD 217/2022 (ESO) y RD 243/2022 (Bachillerato)—, con foco en las materias donde vive lo digital, «Tecnología y Digitalización» (ESO) y «Tecnología e Ingeniería I/II» (Bachillerato), y en la competencia digital transversal. La verificación verbatim contra los PDF consolidados del BOE confirmó que la inteligencia artificial figura de forma nominal y explícita como contenido vinculante: en la ESO, el saber básico C de «Tecnología y Digitalización» incluye «…introducción a la inteligencia artificial» (RD 217/2022, p. 178) y el criterio de evaluación 5.2 cita «módulos de inteligencia artificial» (p. 177); en Bachillerato, los saberes básicos de «Tecnología e Ingeniería II» listan «Inteligencia artificial, big data, bases de datos distribuidas y ciberseguridad» (RD 243/2022, p. 318) y el criterio 5.1 de «Tecnología e Ingeniería I» menciona «…tecnologías emergentes, tales como inteligencia artificial, internet de las cosas, big data…» (p. 316). Las TIC están a su vez plenamente implementadas (competencia digital clave y materias de tecnología de oferta obligatoria). En consecuencia, España se clasifica en la categoría 5 de la escala —«Tiene implementado IA»— con 100 puntos, por encima de la categoría 4 (TIC implementado) al constatarse la IA como contenido nominal de normas curriculares vinculantes en vigor, y no como una mera estrategia no curricular.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>Fuentes</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>RD 217/2022 (ESO) — BOE, PDF consolidado</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>RD 243/2022 (Bachillerato) — BOE, PDF consolidado</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Educagob — Tecnología e Ingeniería (Bachillerato)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>DOG Galicia — Intelixencia Artificial para a Sociedade (4.º ESO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>Alemania (DE)</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Categoría 5 — 100 puntos</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="170" customHeight="1">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>Análisis</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>Para el subindicador «Educación Temprana en IA» del ILIA 2026 se examinó si la base curricular oficial vigente de Alemania incorpora contenidos de inteligencia artificial o de TIC en la educación secundaria (Sekundarstufe I y II), teniendo presente que la competencia curricular corresponde a los Länder y que los documentos de la KMK son coordinadores pero no vinculantes. Se revisó una muestra de currículos de Land con rango normativo, con foco en la asignatura Informatik: el LehrplanPLUS de Baviera (Gymnasium, Jahrgangsstufe 11) y los Kernlehrpläne de Renania del Norte-Westfalia (NRW). La verificación verbatim confirmó que la inteligencia artificial («Künstliche Intelligenz») es contenido vinculante: en Baviera, el plan de Informatik de 11.º contiene un Lernbereich propio titulado «Künstliche Intelligenz (ca. 16 Std.)», cuyas competencias exigen «…diskutieren Ansätze zur Definition des Begriffs Künstliche Intelligenz (KI), beschreiben verschiedene Grundideen von Verfahren der KI (u. a. maschinelles Lernen)…»; en NRW, el Kernlehrplan de Informatik como Pflichtfach de Klasse 5/6 (2021) contiene el Inhaltsfeld «Automaten und künstliche Intelligenz» (p. 14), con los focos «Maschinelles Lernen mit Entscheidungsbäumen» y «…mit neuronalen Netzen» (p. 18). Se constató, además, que el Kernlehrplan GOSt de NRW de 2014 (secundaria superior) no menciona la IA, por lo que la cita vinculante de NRW corresponde al plan de Klasse 5/6. Las TIC/Informatik están implementadas como Pflichtfach en 9 de los 16 Länder en Sek I. En consecuencia, Alemania se clasifica en la categoría 5 —«Tiene implementado IA»— con 100 puntos, con la IA como contenido sustantivo (un módulo dedicado de ~16 h en Baviera) de currículos de Land vigentes; el carácter federal implica que la obligatoriedad varía por Land, lo que se documenta como limitación.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>Fuentes</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>LehrplanPLUS Bayern — Gymnasium 11, Informatik (NTG)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>KLP NRW — Sek I, Klasse 5/6, Informatik (2021, PDF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>Informatik-Monitor 2024/25</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>Estonia (EE)</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>Categoría 5 — 100 puntos</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="170" customHeight="1">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>Análisis</t>
+        </is>
+      </c>
+      <c r="B17" s="15" t="inlineStr">
+        <is>
+          <t>Para el subindicador «Educación Temprana en IA» del ILIA 2026 se examinó si la base curricular oficial vigente de Estonia incorpora contenidos de inteligencia artificial o de TIC en la educación secundaria (põhikool, 7.º–9.º, y gümnaasium, 10.º–12.º). Se revisaron los currículos nacionales (reglamentos del Gobierno consolidados en 2024) y, en particular, el Anexo 10 del Põhikooli riiklik õppekava, correspondiente a la asignatura electiva (valikõppeaine) «Informaatika». La verificación verbatim confirmó que la inteligencia artificial («tehisintellekt») es contenido del currículo nacional: en el III kooliaste, dentro del tema «Infoühiskonna tehnoloogiad» (p. 9), el resultado de aprendizaje (õpitulemus) n.º 6 establece que el alumno «kirjeldab tehisintellekti…» (describe la inteligencia artificial y los usos del internet de las cosas y sus riesgos), y los contenidos (õppesisu) incluyen «Uued tehnoloogiatrendid: tehisintellekt…» y «Tehisintellekti ja asjade interneti mõisted, näited, rakendused ja seonduvad riskid». La competencia digital es, además, una competencia general transversal obligatoria (alineada a DigComp 2.1). Conforme a la metodología del ILIA —confirmada con el equipo del índice, los cursos electivos se consideran parte del currículo nacional—, Estonia se clasifica en la categoría 5 —«Tiene implementado IA»— con 100 puntos. Se deja constancia, por transparencia, de que la IA es contenido de una asignatura electiva y aparece como subtema (uno de nueve resultados de aprendizaje del tema), y de que la iniciativa nacional «AI Leap» (2025) para secundaria superior es dotación de herramientas y formación, aún en desarrollo, que no se computa como currículo vigente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>Fuentes</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>Põhikooli riiklik õppekava — Lisa 10, Informaatika (Riigi Teataja, PDF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Gümnaasiumi riiklik õppekava (EN)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>AI Leap Initiative (Eurydice)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>Singapur (SG)</t>
+        </is>
+      </c>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>Categoría 5 — 100 puntos</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="170" customHeight="1">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t>Análisis</t>
+        </is>
+      </c>
+      <c r="B23" s="15" t="inlineStr">
+        <is>
+          <t>Para el subindicador «Educación Temprana en IA» del ILIA 2026 se examinó si la base curricular oficial vigente de Singapur incorpora contenidos de inteligencia artificial o de TIC en la educación secundaria (Secondary 1–4/5). Se revisó el syllabus oficial del MOE/SEAB de la asignatura «Computing» (Syllabus 7155, examen nacional Singapore-Cambridge GCE O-Level, implementación 2024), cuyos cinco módulos son Computing Fundamentals, Algorithms and Programming, Spreadsheets, Networking e Impact of Computing. La verificación verbatim confirmó que la inteligencia artificial y el aprendizaje automático son contenido examinable del currículo: en el Módulo 5 «Impact of Computing», sección 5.4 «Emerging Technologies» (p. 14), el learning outcome 5.4.1 pide «Describe Artificial Intelligence (AI) as the ability of a computer to perform complex tasks without constant human guidance…» y el 5.4.3 «Define Machine Learning (ML) as a technique used in AI and explain the difference between ML and traditional programming». Conforme a la metodología del ILIA —confirmada con el equipo del índice, los cursos electivos se consideran parte del currículo nacional—, Singapur se clasifica en la categoría 5 —«Tiene implementado IA»— con 100 puntos. Se deja constancia, por transparencia, de que «Computing» es una asignatura electiva y de que la IA/ML aparece como subtema (la sección 5.4, cinco learning outcomes, dentro del Módulo 5), no como un módulo propio; los programas extracurriculares de IA (AI for Fun, Code for Fun) y el uso instrumental de herramientas de IA en el Student Learning Space no se computan como contenido curricular.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
+          <t>Fuentes</t>
+        </is>
+      </c>
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>Computing 7155 — O-Level Syllabus 2025 (SEAB, PDF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="16" t="inlineStr">
+        <is>
+          <t>Computing G3 Syllabus 2024 (MOE, PDF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="16" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence in Education (MOE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>Portugal (PT)</t>
+        </is>
+      </c>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>Categoría 4 — 75 puntos</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="170" customHeight="1">
+      <c r="A29" s="14" t="inlineStr">
+        <is>
+          <t>Análisis</t>
+        </is>
+      </c>
+      <c r="B29" s="15" t="inlineStr">
+        <is>
+          <t>Para el subindicador «Educación Temprana en IA» del ILIA 2026 se examinó si la base curricular oficial vigente de Portugal incorpora contenidos de inteligencia artificial o de TIC en algún nivel del sistema educativo (ensino básico 1.º–9.º y ensino secundário 10.º–12.º). Se revisaron las Aprendizagens Essenciais homologadas y el marco normativo: el Decreto-Lei 55/2018 (currículo de los ensinos básico e secundário), la Portaria 226-A/2018 (matrices curriculares del secundário), el Perfil dos Alunos à Saída da Escolaridade Obrigatória y, en particular, las Aprendizagens Essenciais de la disciplina de informática del secundário, «Aplicações Informáticas B» (12.º ano). La búsqueda de texto completo no halló ninguna mención de «inteligência artificial» como objeto de aprendizaje en el currículo vigente —las Aprendizagens Essenciais de Aplicações Informáticas B se estructuran en solo dos dominios, D1 (Algoritmia e Programação) y D2 (Multimédia)—; la IA aparece únicamente en la revisión curricular del MECI aún no vigente, con nueva versión a consulta pública prevista para 2027 e implementación gradual desde 2027/28, por lo que constituye una propuesta futura y no contenido en vigor. Las TIC, en cambio, están plenamente implementadas: como disciplina obligatoria de TIC en el 3.º ciclo del ensino básico, como «Aplicações Informáticas B» (oferta optativa certificada en el 12.º) y como competencia digital transversal del Perfil dos Alunos. En consecuencia, Portugal se clasifica en la categoría 4 de la escala —«Tiene implementado TIC»— con 75 puntos, sin alcanzar la categoría 5 por la ausencia de IA en el currículo vigente ni quedar por debajo (las TIC están implementadas, no en fase de propuesta); la incorporación de IA prevista para 2027 no altera la clasificación actual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t>Fuentes</t>
+        </is>
+      </c>
+      <c r="B30" s="16" t="inlineStr">
+        <is>
+          <t>DGE — Aplicações Informáticas B (Currículo Nacional)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="16" t="inlineStr">
+        <is>
+          <t>AE Aplicações Informáticas B (12.º), PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="16" t="inlineStr">
+        <is>
+          <t>Decreto-Lei 55/2018</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="16" t="inlineStr">
+        <is>
+          <t>Revisão das Aprendizagens Essenciais (MECI, consulta 2027)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B32" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" r:id="rId17"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>